<commit_message>
Update BOM for revised STM mechanics
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stardance BOM" sheetId="1" r:id="Rae577782e48a4eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcfab602a63b0448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stardance request" sheetId="2" r:id="R07c1fecd159a4ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Self-funded" sheetId="3" r:id="R8c759bdc05734717"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -205,6 +207,25 @@
     <x:xf numFmtId="200" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -407,15 +428,111 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>STM — BOM funding split</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>The grant request and personal workshop purchases are intentionally separate.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+    </x:row>
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>Funding source</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="str">
+        <x:v>Items</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="str">
+        <x:v>Amount</x:v>
+      </x:c>
+      <x:c r="D4" s="45" t="str">
+        <x:v>What it covers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>Stardance</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C5" s="36" t="n">
+        <x:f>'Stardance request'!G37</x:f>
+        <x:v>887.88</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>Build materials, PCBs, mechanics, power, and HOPG reference sample</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="39" t="str">
+        <x:v>Self-funded</x:v>
+      </x:c>
+      <x:c r="B6" s="39" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="n">
+        <x:f>'Self-funded'!G8</x:f>
+        <x:v>179.95</x:v>
+      </x:c>
+      <x:c r="D6" s="39" t="str">
+        <x:v>Soldering, assembly, and inspection tools</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="C7" s="25"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="30" t="str">
+        <x:v>Complete project spend</x:v>
+      </x:c>
+      <x:c r="B8" s="30"/>
+      <x:c r="C8" s="31" t="n">
+        <x:f>SUM(C5:C6)</x:f>
+        <x:v>1067.83</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="str">
+        <x:v>Grant request plus personal workshop purchases</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A8:B8"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="6" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="50" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="46" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -433,7 +550,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="33" t="str">
-        <x:v>Grant-eligible build parts only. Each row lists what to buy and why it is needed.</x:v>
+        <x:v>Build materials and calibration sample only. Prices use the linked product pages.</x:v>
       </x:c>
       <x:c r="B2" s="33"/>
       <x:c r="C2" s="33"/>
@@ -1035,23 +1152,23 @@
         <x:v>Thorlabs KC1T/M kinematic mount</x:v>
       </x:c>
       <x:c r="D23" s="37" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E23" s="37" t="str">
         <x:v>Thorlabs</x:v>
       </x:c>
       <x:c r="F23" s="38" t="n">
-        <x:v>95</x:v>
+        <x:v>116.13</x:v>
       </x:c>
       <x:c r="G23" s="38" t="n">
         <x:f>D23*F23</x:f>
-        <x:v>95</x:v>
+        <x:v>232.26</x:v>
       </x:c>
       <x:c r="H23" s="37" t="str">
         <x:v>https://www.thorlabs.com/thorproduct.cfm?partnumber=KC1T%2FM</x:v>
       </x:c>
       <x:c r="I23" s="37" t="str">
-        <x:v>Holds and finely adjusts the scan head</x:v>
+        <x:v>Two mounts support the revised scan-head design and fine adjustment; price converts the linked EUR listing to USD</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -1355,70 +1472,281 @@
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
-      <x:c r="A34" s="39" t="n">
+      <x:c r="A34" s="37" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B34" s="39" t="str">
+      <x:c r="B34" s="37" t="str">
         <x:v>Noise control</x:v>
       </x:c>
-      <x:c r="C34" s="39" t="str">
+      <x:c r="C34" s="37" t="str">
         <x:v>Copper foil tape with conductive adhesive</x:v>
       </x:c>
-      <x:c r="D34" s="39" t="n">
+      <x:c r="D34" s="37" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E34" s="39" t="str">
+      <x:c r="E34" s="37" t="str">
         <x:v>Adafruit</x:v>
       </x:c>
-      <x:c r="F34" s="40" t="n">
+      <x:c r="F34" s="38" t="n">
         <x:v>5.95</x:v>
       </x:c>
-      <x:c r="G34" s="40" t="n">
+      <x:c r="G34" s="38" t="n">
         <x:f>D34*F34</x:f>
         <x:v>23.8</x:v>
       </x:c>
-      <x:c r="H34" s="39" t="str">
+      <x:c r="H34" s="37" t="str">
         <x:v>https://www.adafruit.com/product/1128</x:v>
       </x:c>
-      <x:c r="I34" s="39" t="str">
+      <x:c r="I34" s="37" t="str">
         <x:v>Provides grounding and shielding around the preamplifier and scan head</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="34"/>
-      <x:c r="B35" s="34"/>
-      <x:c r="C35" s="34"/>
-      <x:c r="D35" s="34"/>
-      <x:c r="E35" s="34"/>
-      <x:c r="F35" s="41"/>
-      <x:c r="G35" s="41"/>
-      <x:c r="H35" s="34"/>
-      <x:c r="I35" s="34"/>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="39" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B35" s="39" t="str">
+        <x:v>Reference sample</x:v>
+      </x:c>
+      <x:c r="C35" s="39" t="str">
+        <x:v>HOPG graphite calibration sample</x:v>
+      </x:c>
+      <x:c r="D35" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="39" t="str">
+        <x:v>Bruker</x:v>
+      </x:c>
+      <x:c r="F35" s="40" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="G35" s="40" t="n">
+        <x:f>D35*F35</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="H35" s="39" t="str">
+        <x:v>https://store.bruker.com/products/hopg</x:v>
+      </x:c>
+      <x:c r="I35" s="39" t="str">
+        <x:v>Provides a known conductive surface for checking the STM before testing other samples</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="42" t="str">
-        <x:v>Requested from Stardance</x:v>
-      </x:c>
-      <x:c r="B36" s="42"/>
-      <x:c r="C36" s="42"/>
-      <x:c r="D36" s="42"/>
-      <x:c r="E36" s="42"/>
-      <x:c r="F36" s="43"/>
-      <x:c r="G36" s="43" t="n">
-        <x:f>SUM(G5:G34)</x:f>
-        <x:v>500.61999999999995</x:v>
-      </x:c>
-      <x:c r="H36" s="42" t="str">
-        <x:v>Tools are not included.</x:v>
-      </x:c>
-      <x:c r="I36" s="42"/>
+      <x:c r="A36" s="34"/>
+      <x:c r="B36" s="34"/>
+      <x:c r="C36" s="34"/>
+      <x:c r="D36" s="34"/>
+      <x:c r="E36" s="34"/>
+      <x:c r="F36" s="41"/>
+      <x:c r="G36" s="41"/>
+      <x:c r="H36" s="34"/>
+      <x:c r="I36" s="34"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="42" t="str">
+        <x:v>Stardance grant request</x:v>
+      </x:c>
+      <x:c r="B37" s="42"/>
+      <x:c r="C37" s="42"/>
+      <x:c r="D37" s="42"/>
+      <x:c r="E37" s="42"/>
+      <x:c r="F37" s="43"/>
+      <x:c r="G37" s="43" t="n">
+        <x:f>SUM(G5:G35)</x:f>
+        <x:v>887.88</x:v>
+      </x:c>
+      <x:c r="H37" s="42" t="str">
+        <x:v>Only this sheet is requested from Stardance.</x:v>
+      </x:c>
+      <x:c r="I37" s="42"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
     <x:mergeCell ref="A2:I2"/>
-    <x:mergeCell ref="A36:F36"/>
-    <x:mergeCell ref="H36:I36"/>
+    <x:mergeCell ref="A37:F37"/>
+    <x:mergeCell ref="H37:I37"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="6" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="50" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="32" t="str">
+        <x:v>STM — Self-funded workshop equipment</x:v>
+      </x:c>
+      <x:c r="B1" s="32"/>
+      <x:c r="C1" s="32"/>
+      <x:c r="D1" s="32"/>
+      <x:c r="E1" s="32"/>
+      <x:c r="F1" s="32"/>
+      <x:c r="G1" s="32"/>
+      <x:c r="H1" s="32"/>
+      <x:c r="I1" s="32"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="33" t="str">
+        <x:v>These workshop purchases are shown for completeness and are not part of the grant request.</x:v>
+      </x:c>
+      <x:c r="B2" s="33"/>
+      <x:c r="C2" s="33"/>
+      <x:c r="D2" s="33"/>
+      <x:c r="E2" s="33"/>
+      <x:c r="F2" s="33"/>
+      <x:c r="G2" s="33"/>
+      <x:c r="H2" s="33"/>
+      <x:c r="I2" s="33"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34"/>
+      <x:c r="B3" s="34"/>
+      <x:c r="C3" s="34"/>
+      <x:c r="D3" s="34"/>
+      <x:c r="E3" s="34"/>
+      <x:c r="F3" s="34"/>
+      <x:c r="G3" s="34"/>
+      <x:c r="H3" s="34"/>
+      <x:c r="I3" s="34"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="11" t="str">
+        <x:v>#</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Section</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Part</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Qty</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Supplier</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>Unit $</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="str">
+        <x:v>Ext. $</x:v>
+      </x:c>
+      <x:c r="H4" s="11" t="str">
+        <x:v>Purchase link</x:v>
+      </x:c>
+      <x:c r="I4" s="11" t="str">
+        <x:v>Why it is needed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Self-funded tools</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>Adafruit electronics toolkit</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str">
+        <x:v>Adafruit</x:v>
+      </x:c>
+      <x:c r="F5" s="36" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G5" s="36" t="n">
+        <x:f>D5*F5</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H5" s="35" t="str">
+        <x:v>https://www.adafruit.com/product/136</x:v>
+      </x:c>
+      <x:c r="I5" s="35" t="str">
+        <x:v>My own purchase for soldering and basic assembly tools</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="39" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B6" s="39" t="str">
+        <x:v>Self-funded tools</x:v>
+      </x:c>
+      <x:c r="C6" s="39" t="str">
+        <x:v>USB microscope with stand</x:v>
+      </x:c>
+      <x:c r="D6" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="39" t="str">
+        <x:v>Adafruit</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="n">
+        <x:v>79.95</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="n">
+        <x:f>D6*F6</x:f>
+        <x:v>79.95</x:v>
+      </x:c>
+      <x:c r="H6" s="39" t="str">
+        <x:v>https://www.adafruit.com/product/636</x:v>
+      </x:c>
+      <x:c r="I6" s="39" t="str">
+        <x:v>My own purchase for inspecting solder joints and tip preparation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="34"/>
+      <x:c r="D7" s="34"/>
+      <x:c r="E7" s="34"/>
+      <x:c r="F7" s="41"/>
+      <x:c r="G7" s="41"/>
+      <x:c r="H7" s="34"/>
+      <x:c r="I7" s="34"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="42" t="str">
+        <x:v>Self-funded subtotal</x:v>
+      </x:c>
+      <x:c r="B8" s="42"/>
+      <x:c r="C8" s="42"/>
+      <x:c r="D8" s="42"/>
+      <x:c r="E8" s="42"/>
+      <x:c r="F8" s="43"/>
+      <x:c r="G8" s="43" t="n">
+        <x:f>SUM(G5:G6)</x:f>
+        <x:v>179.95</x:v>
+      </x:c>
+      <x:c r="H8" s="42" t="str">
+        <x:v>Paid separately; not requested from Stardance.</x:v>
+      </x:c>
+      <x:c r="I8" s="42"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A8:F8"/>
+    <x:mergeCell ref="H8:I8"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>